<commit_message>
added order and order items for the application and also updated the order auto generated mail.
</commit_message>
<xml_diff>
--- a/daily-orders.xlsx
+++ b/daily-orders.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Serial Number</t>
   </si>
@@ -26,13 +26,10 @@
     <t>Order Date</t>
   </si>
   <si>
-    <t>UserName</t>
+    <t>User Email</t>
   </si>
   <si>
     <t>Grand Total</t>
-  </si>
-  <si>
-    <t/>
   </si>
 </sst>
 </file>
@@ -79,6 +76,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="12.39453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="12.46875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="11.66796875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="9.87890625" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.47265625" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
@@ -101,17 +105,11 @@
       <c r="A2" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="B2" t="s" s="0">
-        <v>6</v>
-      </c>
       <c r="C2" t="n" s="0">
         <v>0.0</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>6</v>
-      </c>
       <c r="E2" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>